<commit_message>
additional easy python tasks
</commit_message>
<xml_diff>
--- a/files/programming-tasks/programmieraufgaben_bechtel.xlsx
+++ b/files/programming-tasks/programmieraufgaben_bechtel.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\hefl\files\programming-tasks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C541143D-68E4-4DCB-A112-816C6FDED0CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB872DDF-2BF3-444C-B676-7EDADE10F757}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25650" yWindow="240" windowWidth="39615" windowHeight="20505" tabRatio="540" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-15" yWindow="90" windowWidth="25860" windowHeight="20805" tabRatio="540" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Aufgaben" sheetId="1" r:id="rId1"/>
@@ -389,14 +389,6 @@
 </t>
   </si>
   <si>
-    <t xml:space="preserve">def berechne_flaeche(seitenlänge):
-#deine Lösung
-def gesamtflaeche_schachbrett():
-#deine Lösung
-print gesamtflaeche_schachbrett()
-</t>
-  </si>
-  <si>
     <t>Wenn wir einer Liste ans Ende neue Elemente hinzufügen möchte, kann man die append()-Funktion verwenden. Man benutzt sie so:
 liste = ["Baum", "Wiese", "Garten"] 
 liste.append("Blumen")
@@ -424,6 +416,14 @@
         self.assertEqual(gesamtflaeche_schachbrett(), 256)
 if __name__ == '__main__':
     unittest.main()
+</t>
+  </si>
+  <si>
+    <t xml:space="preserve">def berechne_flaeche(seitenlänge):
+#deine Lösung
+def gesamtflaeche_schachbrett():
+#deine Lösung
+print (gesamtflaeche_schachbrett())
 </t>
   </si>
 </sst>
@@ -1038,7 +1038,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="3" spans="1:16" s="23" customFormat="1" ht="315" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:16" s="23" customFormat="1" ht="360" x14ac:dyDescent="0.25">
       <c r="A3" s="16">
         <v>2</v>
       </c>
@@ -1155,13 +1155,13 @@
         <v>39</v>
       </c>
       <c r="F5" s="18" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="G5" s="23" t="s">
         <v>45</v>
       </c>
       <c r="H5" s="18" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I5" s="17" t="s">
         <v>19</v>
@@ -1205,7 +1205,7 @@
         <v>69</v>
       </c>
       <c r="G6" s="31" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="H6" s="32" t="s">
         <v>70</v>
@@ -1361,7 +1361,7 @@
         <v>37</v>
       </c>
       <c r="D8" s="14" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
     </row>
     <row r="9" spans="1:4" s="2" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>